<commit_message>
Redesign all config tables: items, recipes, cultivation, meridians, rewards, shop, initial_setup
- items.json: 5 types (0=素材192, 1=发射器96, 2=制作台80, 4=配方产物198, 5=效果道具15)
- recipes.json: 210 recipes (cultivation/spirit/wine/sword/array/talisman/breakthrough)
- cultivation.json: 20 stages (凡人→化神前期), 12 breakthrough pills mapped
- meridians.json: 20 stages with comprehensive item pools from type=0+type=4
- home_meridians.json: 109 stages aligned to cultivation, exp=realm requirement
- rewards.json: 218 entries (qi/stamina/exp rewards)
- shop.json: 16 items (materials + products + effects)
- initial_setup.json: 11 Lv.1 launchers + crafting stations
- effects.json: removed (effect config moved into items)
- New effect type: SWORD_QI=7 for flying swords to spawn sword qi
- Update xlsx_to_json.py and json_to_xlsx.py for new schemas
- Update CONFIG.md documentation

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/xlsx/cultivation.xlsx
+++ b/config/xlsx/cultivation.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -525,7 +525,9 @@
       <c r="D4" s="3" t="n">
         <v>110</v>
       </c>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="n">
+        <v>28049</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -559,7 +561,9 @@
       <c r="D6" s="3" t="n">
         <v>130</v>
       </c>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="n">
+        <v>28050</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -645,7 +649,7 @@
         <v>200</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>31</v>
+        <v>28051</v>
       </c>
     </row>
     <row r="12">
@@ -663,7 +667,9 @@
       <c r="D12" s="3" t="n">
         <v>250</v>
       </c>
-      <c r="E12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="n">
+        <v>28052</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -680,7 +686,9 @@
       <c r="D13" s="3" t="n">
         <v>300</v>
       </c>
-      <c r="E13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="n">
+        <v>28053</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -698,7 +706,7 @@
         <v>400</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>32</v>
+        <v>28054</v>
       </c>
     </row>
     <row r="15">
@@ -716,7 +724,9 @@
       <c r="D15" s="3" t="n">
         <v>500</v>
       </c>
-      <c r="E15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="n">
+        <v>28055</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -733,7 +743,9 @@
       <c r="D16" s="3" t="n">
         <v>600</v>
       </c>
-      <c r="E16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="n">
+        <v>28056</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -751,7 +763,7 @@
         <v>800</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>33</v>
+        <v>28057</v>
       </c>
     </row>
     <row r="18">
@@ -769,7 +781,9 @@
       <c r="D18" s="3" t="n">
         <v>1000</v>
       </c>
-      <c r="E18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="n">
+        <v>28058</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -786,7 +800,9 @@
       <c r="D19" s="3" t="n">
         <v>1200</v>
       </c>
-      <c r="E19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="n">
+        <v>28059</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -804,7 +820,7 @@
         <v>1500</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>34</v>
+        <v>28060</v>
       </c>
     </row>
     <row r="21">
@@ -823,199 +839,6 @@
         <v>1800</v>
       </c>
       <c r="E21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>化神中期</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="n">
-        <v>32500</v>
-      </c>
-      <c r="D22" s="3" t="n">
-        <v>2200</v>
-      </c>
-      <c r="E22" s="3" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>化神后期</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="n">
-        <v>84000</v>
-      </c>
-      <c r="D23" s="3" t="n">
-        <v>2800</v>
-      </c>
-      <c r="E23" s="3" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>合体前期</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="n">
-        <v>25000</v>
-      </c>
-      <c r="D24" s="3" t="n">
-        <v>3500</v>
-      </c>
-      <c r="E24" s="3" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>合体中期</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="n">
-        <v>78000</v>
-      </c>
-      <c r="D25" s="3" t="n">
-        <v>4500</v>
-      </c>
-      <c r="E25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>合体后期</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="n">
-        <v>220000</v>
-      </c>
-      <c r="D26" s="3" t="n">
-        <v>6000</v>
-      </c>
-      <c r="E26" s="3" t="n">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>大乘前期</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="n">
-        <v>58000</v>
-      </c>
-      <c r="D27" s="3" t="n">
-        <v>8000</v>
-      </c>
-      <c r="E27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>大乘中期</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="n">
-        <v>250000</v>
-      </c>
-      <c r="D28" s="3" t="n">
-        <v>10000</v>
-      </c>
-      <c r="E28" s="3" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>大乘后期</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="n">
-        <v>830000</v>
-      </c>
-      <c r="D29" s="3" t="n">
-        <v>15000</v>
-      </c>
-      <c r="E29" s="3" t="n">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>渡劫前期</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="n">
-        <v>130000</v>
-      </c>
-      <c r="D30" s="3" t="n">
-        <v>20000</v>
-      </c>
-      <c r="E30" s="3" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>渡劫中期</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="n">
-        <v>670000</v>
-      </c>
-      <c r="D31" s="3" t="n">
-        <v>30000</v>
-      </c>
-      <c r="E31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>渡劫后期</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="n">
-        <v>2200000</v>
-      </c>
-      <c r="D32" s="3" t="n">
-        <v>50000</v>
-      </c>
-      <c r="E32" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
refactor: remove CultivationPanel, refine home UI and server engine
Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/xlsx/cultivation.xlsx
+++ b/config/xlsx/cultivation.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="cultivation" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cultivation" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -475,6 +475,11 @@
           <t>breakthrough_pill</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>breakthrough_reward_id</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -492,6 +497,9 @@
         <v>400</v>
       </c>
       <c r="E2" s="3" t="inlineStr"/>
+      <c r="F2" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -509,6 +517,9 @@
         <v>400</v>
       </c>
       <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -528,6 +539,9 @@
       <c r="E4" s="3" t="n">
         <v>28049</v>
       </c>
+      <c r="F4" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -545,6 +559,9 @@
         <v>600</v>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -564,6 +581,9 @@
       <c r="E6" s="3" t="n">
         <v>28050</v>
       </c>
+      <c r="F6" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -581,6 +601,9 @@
         <v>1000</v>
       </c>
       <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -598,6 +621,9 @@
         <v>1200</v>
       </c>
       <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -615,6 +641,9 @@
         <v>1200</v>
       </c>
       <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -632,6 +661,9 @@
         <v>1700</v>
       </c>
       <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -651,6 +683,9 @@
       <c r="E11" s="3" t="n">
         <v>28051</v>
       </c>
+      <c r="F11" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -670,6 +705,9 @@
       <c r="E12" s="3" t="n">
         <v>28052</v>
       </c>
+      <c r="F12" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -689,6 +727,9 @@
       <c r="E13" s="3" t="n">
         <v>28053</v>
       </c>
+      <c r="F13" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -708,6 +749,9 @@
       <c r="E14" s="3" t="n">
         <v>28054</v>
       </c>
+      <c r="F14" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -727,6 +771,9 @@
       <c r="E15" s="3" t="n">
         <v>28055</v>
       </c>
+      <c r="F15" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -746,6 +793,9 @@
       <c r="E16" s="3" t="n">
         <v>28056</v>
       </c>
+      <c r="F16" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -765,6 +815,9 @@
       <c r="E17" s="3" t="n">
         <v>28057</v>
       </c>
+      <c r="F17" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -784,6 +837,9 @@
       <c r="E18" s="3" t="n">
         <v>28058</v>
       </c>
+      <c r="F18" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -803,6 +859,9 @@
       <c r="E19" s="3" t="n">
         <v>28059</v>
       </c>
+      <c r="F19" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -821,6 +880,9 @@
       </c>
       <c r="E20" s="3" t="n">
         <v>28060</v>
+      </c>
+      <c r="F20" t="n">
+        <v>220</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Implement merge game systems and UI
</commit_message>
<xml_diff>
--- a/config/xlsx/cultivation.xlsx
+++ b/config/xlsx/cultivation.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cultivation" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="cultivation" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -496,7 +496,9 @@
       <c r="D2" s="3" t="n">
         <v>400</v>
       </c>
-      <c r="E2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="n">
+        <v>14101</v>
+      </c>
       <c r="F2" t="n">
         <v>220</v>
       </c>

</xml_diff>

<commit_message>
Refactor game architecture and update project configuration
</commit_message>
<xml_diff>
--- a/config/xlsx/cultivation.xlsx
+++ b/config/xlsx/cultivation.xlsx
@@ -447,6 +447,7 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -475,7 +476,7 @@
           <t>breakthrough_pill</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>breakthrough_reward_id</t>
         </is>
@@ -499,9 +500,7 @@
       <c r="E2" s="3" t="n">
         <v>14101</v>
       </c>
-      <c r="F2" t="n">
-        <v>220</v>
-      </c>
+      <c r="F2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -519,9 +518,7 @@
         <v>400</v>
       </c>
       <c r="E3" s="3" t="inlineStr"/>
-      <c r="F3" t="n">
-        <v>220</v>
-      </c>
+      <c r="F3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -541,9 +538,7 @@
       <c r="E4" s="3" t="n">
         <v>28049</v>
       </c>
-      <c r="F4" t="n">
-        <v>220</v>
-      </c>
+      <c r="F4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -561,9 +556,7 @@
         <v>600</v>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" t="n">
-        <v>220</v>
-      </c>
+      <c r="F5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -583,9 +576,7 @@
       <c r="E6" s="3" t="n">
         <v>28050</v>
       </c>
-      <c r="F6" t="n">
-        <v>220</v>
-      </c>
+      <c r="F6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -603,9 +594,7 @@
         <v>1000</v>
       </c>
       <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" t="n">
-        <v>220</v>
-      </c>
+      <c r="F7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -623,9 +612,7 @@
         <v>1200</v>
       </c>
       <c r="E8" s="3" t="inlineStr"/>
-      <c r="F8" t="n">
-        <v>220</v>
-      </c>
+      <c r="F8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -643,9 +630,7 @@
         <v>1200</v>
       </c>
       <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" t="n">
-        <v>220</v>
-      </c>
+      <c r="F9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -663,9 +648,7 @@
         <v>1700</v>
       </c>
       <c r="E10" s="3" t="inlineStr"/>
-      <c r="F10" t="n">
-        <v>220</v>
-      </c>
+      <c r="F10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -685,9 +668,7 @@
       <c r="E11" s="3" t="n">
         <v>28051</v>
       </c>
-      <c r="F11" t="n">
-        <v>220</v>
-      </c>
+      <c r="F11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -707,9 +688,7 @@
       <c r="E12" s="3" t="n">
         <v>28052</v>
       </c>
-      <c r="F12" t="n">
-        <v>220</v>
-      </c>
+      <c r="F12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -729,9 +708,7 @@
       <c r="E13" s="3" t="n">
         <v>28053</v>
       </c>
-      <c r="F13" t="n">
-        <v>220</v>
-      </c>
+      <c r="F13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -751,9 +728,7 @@
       <c r="E14" s="3" t="n">
         <v>28054</v>
       </c>
-      <c r="F14" t="n">
-        <v>220</v>
-      </c>
+      <c r="F14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -773,9 +748,7 @@
       <c r="E15" s="3" t="n">
         <v>28055</v>
       </c>
-      <c r="F15" t="n">
-        <v>220</v>
-      </c>
+      <c r="F15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -795,9 +768,7 @@
       <c r="E16" s="3" t="n">
         <v>28056</v>
       </c>
-      <c r="F16" t="n">
-        <v>220</v>
-      </c>
+      <c r="F16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -817,9 +788,7 @@
       <c r="E17" s="3" t="n">
         <v>28057</v>
       </c>
-      <c r="F17" t="n">
-        <v>220</v>
-      </c>
+      <c r="F17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -839,9 +808,7 @@
       <c r="E18" s="3" t="n">
         <v>28058</v>
       </c>
-      <c r="F18" t="n">
-        <v>220</v>
-      </c>
+      <c r="F18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -861,9 +828,7 @@
       <c r="E19" s="3" t="n">
         <v>28059</v>
       </c>
-      <c r="F19" t="n">
-        <v>220</v>
-      </c>
+      <c r="F19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -883,9 +848,7 @@
       <c r="E20" s="3" t="n">
         <v>28060</v>
       </c>
-      <c r="F20" t="n">
-        <v>220</v>
-      </c>
+      <c r="F20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -903,6 +866,7 @@
         <v>3100</v>
       </c>
       <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update merge game systems and configuration
</commit_message>
<xml_diff>
--- a/config/xlsx/cultivation.xlsx
+++ b/config/xlsx/cultivation.xlsx
@@ -2,86 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cultivation" sheetId="1" r:id="Raac4505f68764f7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cultivation" sheetId="1" r:id="R5876b4d3f21b4c34"/>
   </x:sheets>
 </x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:si>
-    <x:t xml:space="preserve">stage_index</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">name</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">exp</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">max_qi</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">凡人</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">练气一层</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">练气二层</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">练气三层</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">练气四层</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">练气五层</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">练气六层</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">练气七层</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">练气八层</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">练气九层</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">筑基前期</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">筑基中期</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">筑基后期</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">金丹前期</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">金丹中期</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">金丹后期</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">元婴前期</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">元婴中期</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">元婴后期</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">化神前期</x:t>
-  </x:si>
-</x:sst>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -209,7 +136,7 @@
       <x:name val="宋体"/>
     </x:font>
   </x:fonts>
-  <x:fills count="34">
+  <x:fills count="37">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -376,8 +303,23 @@
         <x:fgColor theme="9" tint="0.39998"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4472C4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4472C4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4472C4"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="10">
+  <x:borders count="11">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -472,6 +414,20 @@
         <x:color theme="4"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="49">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -620,7 +576,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="4">
+  <x:cellXfs count="21">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
@@ -630,6 +586,37 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="35" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="35" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="35" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="36" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="36" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="36" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="49">
@@ -904,399 +891,418 @@
   <x:cols>
     <x:col min="1" max="6" width="16" customWidth="1"/>
     <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="1" t="s">
+      <x:c r="A1" s="20" t="str">
+        <x:v>stage_index</x:v>
+      </x:c>
+      <x:c r="B1" s="20" t="str">
+        <x:v>name</x:v>
+      </x:c>
+      <x:c r="C1" s="20" t="str">
+        <x:v>exp</x:v>
+      </x:c>
+      <x:c r="D1" s="20" t="str">
+        <x:v>max_qi</x:v>
+      </x:c>
+      <x:c r="E1" s="20" t="str">
+        <x:v>breakthrough_items</x:v>
+      </x:c>
+      <x:c r="F1" s="20" t="str">
+        <x:v>breakthrough_reward_id</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="10" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="B1" s="1" t="s">
+      <x:c r="B2" s="10" t="str">
+        <x:v>凡人</x:v>
+      </x:c>
+      <x:c r="C2" s="10" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D2" s="10" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="E2" s="10" t="str">
+        <x:v>14101:1</x:v>
+      </x:c>
+      <x:c r="F2" s="10" t="n">
+        <x:v>313</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C1" s="1" t="s">
+      <x:c r="B3" s="10" t="str">
+        <x:v>练气一层</x:v>
+      </x:c>
+      <x:c r="C3" s="10" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="D3" s="10" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="E3" s="10" t="str"/>
+      <x:c r="F3" s="10" t="n">
+        <x:v>313</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="10" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D1" s="1" t="s">
+      <x:c r="B4" s="10" t="str">
+        <x:v>练气二层</x:v>
+      </x:c>
+      <x:c r="C4" s="10" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="D4" s="10" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="E4" s="10" t="str">
+        <x:v>28049:1</x:v>
+      </x:c>
+      <x:c r="F4" s="10" t="n">
+        <x:v>311</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="10" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E1" s="1" t="str">
-        <x:v>breakthrough_items</x:v>
-      </x:c>
-      <x:c r="F1" s="1" t="str">
-        <x:v>breakthrough_reward_id</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="2">
+      <x:c r="B5" s="10" t="str">
+        <x:v>练气三层</x:v>
+      </x:c>
+      <x:c r="C5" s="10" t="n">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="D5" s="10" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="E5" s="10" t="str"/>
+      <x:c r="F5" s="10" t="n">
+        <x:v>313</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="10" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B6" s="10" t="str">
+        <x:v>练气四层</x:v>
+      </x:c>
+      <x:c r="C6" s="10" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="D6" s="10" t="n">
+        <x:v>8000</x:v>
+      </x:c>
+      <x:c r="E6" s="10" t="str">
+        <x:v>28050:1</x:v>
+      </x:c>
+      <x:c r="F6" s="10" t="n">
+        <x:v>313</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B7" s="10" t="str">
+        <x:v>练气五层</x:v>
+      </x:c>
+      <x:c r="C7" s="10" t="n">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="D7" s="10" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="E7" s="10" t="str"/>
+      <x:c r="F7" s="10" t="n">
+        <x:v>313</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="10" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B8" s="10" t="str">
+        <x:v>练气六层</x:v>
+      </x:c>
+      <x:c r="C8" s="10" t="n">
+        <x:v>264</x:v>
+      </x:c>
+      <x:c r="D8" s="10" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="E8" s="10" t="str">
+        <x:v>28050:1</x:v>
+      </x:c>
+      <x:c r="F8" s="10" t="n">
+        <x:v>312</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="10" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B9" s="10" t="str">
+        <x:v>练气七层</x:v>
+      </x:c>
+      <x:c r="C9" s="10" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="D9" s="10" t="n">
+        <x:v>15000</x:v>
+      </x:c>
+      <x:c r="E9" s="10" t="str"/>
+      <x:c r="F9" s="10" t="n">
+        <x:v>313</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="10" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B10" s="10" t="str">
+        <x:v>练气八层</x:v>
+      </x:c>
+      <x:c r="C10" s="10" t="n">
+        <x:v>348</x:v>
+      </x:c>
+      <x:c r="D10" s="10" t="n">
+        <x:v>17000</x:v>
+      </x:c>
+      <x:c r="E10" s="10" t="str"/>
+      <x:c r="F10" s="10" t="n">
+        <x:v>313</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="10" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B11" s="10" t="str">
+        <x:v>练气九层</x:v>
+      </x:c>
+      <x:c r="C11" s="10" t="n">
+        <x:v>384</x:v>
+      </x:c>
+      <x:c r="D11" s="10" t="n">
+        <x:v>20000</x:v>
+      </x:c>
+      <x:c r="E11" s="10" t="str">
+        <x:v>28051:1</x:v>
+      </x:c>
+      <x:c r="F11" s="10" t="n">
+        <x:v>301</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="10" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B12" s="10" t="str">
+        <x:v>筑基前期</x:v>
+      </x:c>
+      <x:c r="C12" s="10" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="D12" s="10" t="n">
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="E12" s="10" t="str">
+        <x:v>28052:1</x:v>
+      </x:c>
+      <x:c r="F12" s="10" t="n">
+        <x:v>302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="10" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B13" s="10" t="str">
+        <x:v>筑基中期</x:v>
+      </x:c>
+      <x:c r="C13" s="10" t="n">
+        <x:v>2150</x:v>
+      </x:c>
+      <x:c r="D13" s="10" t="n">
+        <x:v>200000</x:v>
+      </x:c>
+      <x:c r="E13" s="10" t="str">
+        <x:v>28053:1</x:v>
+      </x:c>
+      <x:c r="F13" s="10" t="n">
+        <x:v>303</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="10" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B14" s="10" t="str">
+        <x:v>筑基后期</x:v>
+      </x:c>
+      <x:c r="C14" s="10" t="n">
+        <x:v>3900</x:v>
+      </x:c>
+      <x:c r="D14" s="10" t="n">
+        <x:v>400000</x:v>
+      </x:c>
+      <x:c r="E14" s="10" t="str">
+        <x:v>28054:1</x:v>
+      </x:c>
+      <x:c r="F14" s="10" t="n">
+        <x:v>304</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="10" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B15" s="10" t="str">
+        <x:v>金丹前期</x:v>
+      </x:c>
+      <x:c r="C15" s="10" t="n">
+        <x:v>2200</x:v>
+      </x:c>
+      <x:c r="D15" s="10" t="n">
+        <x:v>1000000</x:v>
+      </x:c>
+      <x:c r="E15" s="10" t="str">
+        <x:v>28055:1</x:v>
+      </x:c>
+      <x:c r="F15" s="10" t="n">
+        <x:v>305</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="10" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B16" s="10" t="str">
+        <x:v>金丹中期</x:v>
+      </x:c>
+      <x:c r="C16" s="10" t="n">
+        <x:v>6300</x:v>
+      </x:c>
+      <x:c r="D16" s="10" t="n">
+        <x:v>4000000</x:v>
+      </x:c>
+      <x:c r="E16" s="10" t="str">
+        <x:v>28056:1</x:v>
+      </x:c>
+      <x:c r="F16" s="10" t="n">
+        <x:v>306</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="10" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B17" s="10" t="str">
+        <x:v>金丹后期</x:v>
+      </x:c>
+      <x:c r="C17" s="10" t="n">
+        <x:v>13600</x:v>
+      </x:c>
+      <x:c r="D17" s="10" t="n">
+        <x:v>8000000</x:v>
+      </x:c>
+      <x:c r="E17" s="10" t="str">
+        <x:v>28057:1</x:v>
+      </x:c>
+      <x:c r="F17" s="10" t="n">
+        <x:v>307</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="10" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B18" s="10" t="str">
+        <x:v>元婴前期</x:v>
+      </x:c>
+      <x:c r="C18" s="10" t="n">
+        <x:v>4700</x:v>
+      </x:c>
+      <x:c r="D18" s="10" t="n">
+        <x:v>100000000</x:v>
+      </x:c>
+      <x:c r="E18" s="10" t="str">
+        <x:v>28058:1</x:v>
+      </x:c>
+      <x:c r="F18" s="10" t="n">
+        <x:v>308</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="10" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B19" s="10" t="str">
+        <x:v>元婴中期</x:v>
+      </x:c>
+      <x:c r="C19" s="10" t="n">
+        <x:v>13700</x:v>
+      </x:c>
+      <x:c r="D19" s="10" t="n">
+        <x:v>500000000</x:v>
+      </x:c>
+      <x:c r="E19" s="10" t="str">
+        <x:v>28059:1</x:v>
+      </x:c>
+      <x:c r="F19" s="10" t="n">
+        <x:v>309</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="10" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B20" s="10" t="str">
+        <x:v>元婴后期</x:v>
+      </x:c>
+      <x:c r="C20" s="10" t="n">
+        <x:v>31000</x:v>
+      </x:c>
+      <x:c r="D20" s="10" t="n">
+        <x:v>1000000000</x:v>
+      </x:c>
+      <x:c r="E20" s="10" t="str">
+        <x:v>28060:1</x:v>
+      </x:c>
+      <x:c r="F20" s="10" t="n">
+        <x:v>310</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="10" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B21" s="10" t="str">
+        <x:v>化神前期</x:v>
+      </x:c>
+      <x:c r="C21" s="10" t="n">
+        <x:v>99999999</x:v>
+      </x:c>
+      <x:c r="D21" s="10" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="B2" s="2" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C2" s="3">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="D2" s="3">
-        <x:v>1000</x:v>
-      </x:c>
-      <x:c r="E2" s="3" t="str">
-        <x:v>14101:1</x:v>
-      </x:c>
-      <x:c r="F2" s="3" t="str"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="2">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B3" s="2" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C3" s="3">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="D3" s="3">
-        <x:v>4000</x:v>
-      </x:c>
-      <x:c r="E3" s="3" t="str"/>
-      <x:c r="F3" s="3" t="str"/>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="2">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B4" s="2" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C4" s="3">
-        <x:v>90</x:v>
-      </x:c>
-      <x:c r="D4" s="3">
-        <x:v>6000</x:v>
-      </x:c>
-      <x:c r="E4" s="3" t="str">
-        <x:v>28049:1</x:v>
-      </x:c>
-      <x:c r="F4" s="3" t="n">
-        <x:v>311</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="2">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B5" s="2" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C5" s="3">
-        <x:v>108</x:v>
-      </x:c>
-      <x:c r="D5" s="3">
-        <x:v>6000</x:v>
-      </x:c>
-      <x:c r="E5" s="3" t="str"/>
-      <x:c r="F5" s="3" t="str"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="2">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B6" s="2" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C6" s="3">
-        <x:v>157</x:v>
-      </x:c>
-      <x:c r="D6" s="3">
-        <x:v>8000</x:v>
-      </x:c>
-      <x:c r="E6" s="3" t="str">
-        <x:v>28050:1</x:v>
-      </x:c>
-      <x:c r="F6" s="3" t="str"/>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="2">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B7" s="2" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C7" s="3">
-        <x:v>214</x:v>
-      </x:c>
-      <x:c r="D7" s="3">
-        <x:v>10000</x:v>
-      </x:c>
-      <x:c r="E7" s="3" t="str"/>
-      <x:c r="F7" s="3" t="str"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="2">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B8" s="2" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C8" s="3">
-        <x:v>320</x:v>
-      </x:c>
-      <x:c r="D8" s="3">
-        <x:v>12000</x:v>
-      </x:c>
-      <x:c r="E8" s="3" t="str">
-        <x:v>28050:1</x:v>
-      </x:c>
-      <x:c r="F8" s="3" t="n">
-        <x:v>312</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="2">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="B9" s="2" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C9" s="3">
-        <x:v>400</x:v>
-      </x:c>
-      <x:c r="D9" s="3">
-        <x:v>15000</x:v>
-      </x:c>
-      <x:c r="E9" s="3" t="str"/>
-      <x:c r="F9" s="3" t="str"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="2">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="B10" s="2" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C10" s="3">
-        <x:v>500</x:v>
-      </x:c>
-      <x:c r="D10" s="3">
-        <x:v>17000</x:v>
-      </x:c>
-      <x:c r="E10" s="3" t="str"/>
-      <x:c r="F10" s="3" t="str"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="2">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B11" s="2" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C11" s="3">
-        <x:v>600</x:v>
-      </x:c>
-      <x:c r="D11" s="3">
-        <x:v>20000</x:v>
-      </x:c>
-      <x:c r="E11" s="3" t="str">
-        <x:v>28051:1</x:v>
-      </x:c>
-      <x:c r="F11" s="3" t="n">
-        <x:v>301</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="2">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B12" s="2" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C12" s="3">
-        <x:v>900</x:v>
-      </x:c>
-      <x:c r="D12" s="3">
-        <x:v>100000</x:v>
-      </x:c>
-      <x:c r="E12" s="3" t="str">
-        <x:v>28052:1</x:v>
-      </x:c>
-      <x:c r="F12" s="3" t="n">
-        <x:v>302</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="2">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B13" s="2" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C13" s="3">
-        <x:v>2150</x:v>
-      </x:c>
-      <x:c r="D13" s="3">
-        <x:v>200000</x:v>
-      </x:c>
-      <x:c r="E13" s="3" t="str">
-        <x:v>28053:1</x:v>
-      </x:c>
-      <x:c r="F13" s="3" t="n">
-        <x:v>303</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="2">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B14" s="2" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C14" s="3">
-        <x:v>3900</x:v>
-      </x:c>
-      <x:c r="D14" s="3">
-        <x:v>400000</x:v>
-      </x:c>
-      <x:c r="E14" s="3" t="str">
-        <x:v>28054:1</x:v>
-      </x:c>
-      <x:c r="F14" s="3" t="n">
-        <x:v>304</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="2">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B15" s="2" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C15" s="3">
-        <x:v>2200</x:v>
-      </x:c>
-      <x:c r="D15" s="3">
-        <x:v>1000000</x:v>
-      </x:c>
-      <x:c r="E15" s="3" t="str">
-        <x:v>28055:1</x:v>
-      </x:c>
-      <x:c r="F15" s="3" t="n">
-        <x:v>305</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="2">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B16" s="2" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C16" s="3">
-        <x:v>6300</x:v>
-      </x:c>
-      <x:c r="D16" s="3">
-        <x:v>4000000</x:v>
-      </x:c>
-      <x:c r="E16" s="3" t="str">
-        <x:v>28056:1</x:v>
-      </x:c>
-      <x:c r="F16" s="3" t="n">
-        <x:v>306</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="2">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B17" s="2" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C17" s="3">
-        <x:v>13600</x:v>
-      </x:c>
-      <x:c r="D17" s="3">
-        <x:v>8000000</x:v>
-      </x:c>
-      <x:c r="E17" s="3" t="str">
-        <x:v>28057:1</x:v>
-      </x:c>
-      <x:c r="F17" s="3" t="n">
-        <x:v>307</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="2">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B18" s="2" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="C18" s="3">
-        <x:v>4700</x:v>
-      </x:c>
-      <x:c r="D18" s="3">
-        <x:v>100000000</x:v>
-      </x:c>
-      <x:c r="E18" s="3" t="str">
-        <x:v>28058:1</x:v>
-      </x:c>
-      <x:c r="F18" s="3" t="n">
-        <x:v>308</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="2">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B19" s="2" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="C19" s="3">
-        <x:v>13700</x:v>
-      </x:c>
-      <x:c r="D19" s="3">
-        <x:v>500000000</x:v>
-      </x:c>
-      <x:c r="E19" s="3" t="str">
-        <x:v>28059:1</x:v>
-      </x:c>
-      <x:c r="F19" s="3" t="n">
-        <x:v>309</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="2">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="B20" s="2" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="C20" s="3">
-        <x:v>31000</x:v>
-      </x:c>
-      <x:c r="D20" s="3">
-        <x:v>1000000000</x:v>
-      </x:c>
-      <x:c r="E20" s="3" t="str">
-        <x:v>28060:1</x:v>
-      </x:c>
-      <x:c r="F20" s="3" t="n">
-        <x:v>310</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="2">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="B21" s="2" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="C21" s="3">
-        <x:v>99999999</x:v>
-      </x:c>
-      <x:c r="D21" s="3">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E21" s="3" t="str"/>
-      <x:c r="F21" s="3" t="str"/>
+      <x:c r="E21" s="10" t="str"/>
+      <x:c r="F21" s="10"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>